<commit_message>
Verifica settimanale: 73 duplicati marcati, 53 upgrade doppio controllo
Deduplica globale ricostruita su 294 file / 2164 righe (schema verifica),
con guardia anti-filiale rafforzata (indicatori anche in provincia_area,
qualificatori geografici nudi tra parentesi, blocco su domini diversi per
match-per-nome) e rivalidazione diretta contro la riga canonica per
eliminare falsi positivi da transitività nell'union-find.

Doppio controllo via 9 agenti paralleli su 139 righe candidate nei 29 file
nuovi (Malesia: Kelantan/Melaka/Negeri Sembilan/Pahang/Perak): 53 promosse
a "VERIFICATA AI - doppio controllo", 86 lasciate invariate per esito non
confermato o settore incoerente.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uy819AamPSHFihS6HWfy2z
</commit_message>
<xml_diff>
--- a/output/2026-09-14_17_Croazia_Licko-senjska_ATEX_Equipment-Services.xlsx
+++ b/output/2026-09-14_17_Croazia_Licko-senjska_ATEX_Equipment-Services.xlsx
@@ -474,7 +474,6 @@
           <t>VRKLJAN d.o.o.</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Ličko-senjska županija (Gospić)</t>
@@ -490,10 +489,9 @@
           <t>053 572 817</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>SCARTATA: rivenditore generico di materiale edile/ferramenta/vernici/generi alimentari (attivo dal 1990). Nessuna evidenza di prodotti/attrezzature ATEX. Fuori target settore.</t>
+          <t>SCARTATA: rivenditore generico di materiale edile/ferramenta/vernici/generi alimentari (attivo dal 1990). Nessuna evidenza di prodotti/attrezzature ATEX. Fuori target settore. [DUPLICATO — vedi anche: 2026-09-14_03_Croazia_Licko-senjska_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -508,7 +506,6 @@
           <t>MARTINČIĆ d.o.o.</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Ličko-senjska županija (Gospić)</t>
@@ -519,11 +516,9 @@
           <t>ATEX Equipment/Services</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>SCARTATA: rivenditore generico di materiale elettrico/edile/vernici, dealer Saint-Gobain (attivo dal 1996/97). Nessuna evidenza di prodotti antideflagranti/certificati ATEX. Fuori target settore.</t>
+          <t>SCARTATA: rivenditore generico di materiale elettrico/edile/vernici, dealer Saint-Gobain (attivo dal 1996/97). Nessuna evidenza di prodotti antideflagranti/certificati ATEX. Fuori target settore. [DUPLICATO — vedi anche: 2026-09-14_03_Croazia_Licko-senjska_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -538,7 +533,6 @@
           <t>ŠANTIĆ d.o.o.</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Ličko-senjska županija (Otočac)</t>
@@ -549,8 +543,6 @@
           <t>ATEX Equipment/Services</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>SCARTATA: attività reale = taglio/lavorazione legname (Sječa drva), difforme dalla descrizione iniziale (idraulica-pneumatica/metalli). Potenziale cliente finale (utilizzatore di impianti aspirazione, non venditore), non distributore.</t>

</xml_diff>